<commit_message>
Improvements made to DCF logic and exporting
</commit_message>
<xml_diff>
--- a/data/AAPL_valuation_20260601.xlsx
+++ b/data/AAPL_valuation_20260601.xlsx
@@ -743,7 +743,7 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>3993054000000</v>
+        <v>3246372121322.635</v>
       </c>
     </row>
     <row r="14">
@@ -753,7 +753,7 @@
         </is>
       </c>
       <c r="C14" s="8" t="n">
-        <v>4026817000000</v>
+        <v>3280135121322.635</v>
       </c>
     </row>
     <row r="15">
@@ -763,7 +763,7 @@
         </is>
       </c>
       <c r="C15" s="9" t="n">
-        <v>274.1689518521918</v>
+        <v>223.3305382754143</v>
       </c>
     </row>
     <row r="16">
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="C16" s="10" t="n">
-        <v>-0.1172308094358399</v>
+        <v>-0.3715544786904796</v>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
@@ -801,7 +801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G29"/>
+  <dimension ref="B1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -842,265 +842,275 @@
     <row r="5">
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Base FCF (3yr avg)</t>
+          <t>Base FCFF (3yr avg)</t>
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>102386000000</v>
+        <v>103455910666.6667</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Discount Rate (WACC)</t>
+          <t>Tax Rate</t>
         </is>
       </c>
       <c r="C6" s="12" t="n">
-        <v>0.05</v>
+        <v>0.156</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Growth Rate</t>
+          <t>Discount Rate (WACC)</t>
         </is>
       </c>
       <c r="C7" s="12" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Terminal Growth</t>
+          <t>Growth Rate</t>
         </is>
       </c>
       <c r="C8" s="12" t="n">
-        <v>0.02</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t>Terminal Growth</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="5" t="inlineStr">
+        <is>
           <t>Projection Years</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C10" s="13" t="n">
         <v>5</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="B11" s="14" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>Cash Flow</t>
         </is>
       </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>Year 1</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Year 2</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
         <is>
           <t>Year 3</t>
         </is>
       </c>
-      <c r="F11" s="15" t="inlineStr">
+      <c r="F12" s="15" t="inlineStr">
         <is>
           <t>Year 4</t>
         </is>
       </c>
-      <c r="G11" s="15" t="inlineStr">
+      <c r="G12" s="15" t="inlineStr">
         <is>
           <t>Year 5</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="16" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Projected FCF</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n">
-        <v>107505300000</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <v>112880565000</v>
-      </c>
-      <c r="E12" s="17" t="n">
-        <v>118524593250</v>
-      </c>
-      <c r="F12" s="17" t="n">
-        <v>124450822912.5</v>
-      </c>
-      <c r="G12" s="17" t="n">
-        <v>130673364058.125</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="18" t="inlineStr">
+      <c r="C13" s="17" t="n">
+        <v>115870619946.6667</v>
+      </c>
+      <c r="D13" s="17" t="n">
+        <v>129775094340.2667</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>145348105661.0987</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>162789878340.4306</v>
+      </c>
+      <c r="G13" s="17" t="n">
+        <v>182324663741.2823</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="18" t="inlineStr">
         <is>
           <t>Present Value of FCF</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n">
-        <v>102386000000</v>
-      </c>
-      <c r="D13" s="19" t="n">
-        <v>102386000000</v>
-      </c>
-      <c r="E13" s="19" t="n">
-        <v>102386000000</v>
-      </c>
-      <c r="F13" s="19" t="n">
-        <v>102386000000</v>
-      </c>
-      <c r="G13" s="19" t="n">
-        <v>102386000000</v>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="B15" s="3" t="inlineStr">
+      <c r="C14" s="19" t="n">
+        <v>108290299015.5763</v>
+      </c>
+      <c r="D14" s="19" t="n">
+        <v>113350593362.0986</v>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>118647350061.2621</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>124191618755.7136</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>129994965426.5413</v>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Terminal &amp; Totals</t>
         </is>
       </c>
-      <c r="C15" s="4" t="n"/>
-      <c r="D15" s="4" t="n"/>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="n"/>
-      <c r="G15" s="4" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Terminal Value</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n">
-        <v>4442894377976.251</v>
-      </c>
+      <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
+      <c r="E16" s="4" t="n"/>
+      <c r="F16" s="4" t="n"/>
+      <c r="G16" s="4" t="n"/>
     </row>
     <row r="17">
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>PV of Terminal Value</t>
+          <t>Terminal Value</t>
         </is>
       </c>
       <c r="C17" s="8" t="n">
-        <v>3481124000000</v>
+        <v>3719423140322.158</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Sum PV of FCFs</t>
+          <t>PV of Terminal Value</t>
         </is>
       </c>
       <c r="C18" s="8" t="n">
-        <v>511930000000</v>
+        <v>2651897294701.443</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
+          <t>Sum PV of FCFs</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>594474826621.192</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="5" t="inlineStr">
+        <is>
           <t>Enterprise Value</t>
         </is>
       </c>
-      <c r="C19" s="20" t="n">
-        <v>3993054000000</v>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="B21" s="3" t="inlineStr">
+      <c r="C20" s="20" t="n">
+        <v>3246372121322.635</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Equity Bridge</t>
         </is>
       </c>
-      <c r="C21" s="4" t="n"/>
-      <c r="D21" s="4" t="n"/>
-      <c r="E21" s="4" t="n"/>
-      <c r="F21" s="4" t="n"/>
-      <c r="G21" s="4" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Enterprise Value</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n">
-        <v>3993054000000</v>
-      </c>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+      <c r="E22" s="4" t="n"/>
+      <c r="F22" s="4" t="n"/>
+      <c r="G22" s="4" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>Less: Total Debt</t>
-        </is>
-      </c>
-      <c r="C23" s="21" t="n">
-        <v>-98657000000</v>
+          <t>Enterprise Value</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="n">
+        <v>3246372121322.635</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>Add: Cash &amp; ST Investments</t>
-        </is>
-      </c>
-      <c r="C24" s="22" t="n">
-        <v>54697000000</v>
+          <t>Less: Total Debt</t>
+        </is>
+      </c>
+      <c r="C24" s="21" t="n">
+        <v>-98657000000</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Add: LT Investments (non-op)</t>
+          <t>Add: Cash &amp; ST Investments</t>
         </is>
       </c>
       <c r="C25" s="22" t="n">
-        <v>77723000000</v>
+        <v>54697000000</v>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Equity Value</t>
-        </is>
-      </c>
-      <c r="C26" s="20" t="n">
-        <v>4026817000000</v>
+          <t>Add: LT Investments (non-op)</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="n">
+        <v>77723000000</v>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>Shares Outstanding</t>
-        </is>
-      </c>
-      <c r="C27" s="23" t="n">
-        <v>14687356000</v>
+          <t>Equity Value</t>
+        </is>
+      </c>
+      <c r="C27" s="20" t="n">
+        <v>3280135121322.635</v>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="5" t="inlineStr">
         <is>
+          <t>Shares Outstanding</t>
+        </is>
+      </c>
+      <c r="C28" s="23" t="n">
+        <v>14687356000</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="5" t="inlineStr">
+        <is>
           <t>Intrinsic Value / Share</t>
         </is>
       </c>
-      <c r="C28" s="9" t="n">
-        <v>274.1689518521918</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="24" t="inlineStr">
+      <c r="C29" s="9" t="n">
+        <v>223.3305382754143</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="24" t="inlineStr">
         <is>
           <t>Net debt source: balance sheet (annual)</t>
         </is>
@@ -1109,11 +1119,11 @@
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B22:G22"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="B4:G4"/>
-    <mergeCell ref="B29:G29"/>
-    <mergeCell ref="B21:G21"/>
-    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B30:G30"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1159,138 +1169,138 @@
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>10%</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>11%</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>12%</t>
         </is>
       </c>
       <c r="F4" s="15" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>13%</t>
         </is>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>14%</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>3%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="C5" s="26" t="n">
-        <v>748.2</v>
+        <v>345.09</v>
       </c>
       <c r="D5" s="26" t="n">
-        <v>784.42</v>
+        <v>360.23</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>822.05</v>
+        <v>375.92</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>861.13</v>
+        <v>392.16</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>901.6900000000001</v>
+        <v>408.98</v>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>4%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="C6" s="26" t="n">
-        <v>374.92</v>
+        <v>257.88</v>
       </c>
       <c r="D6" s="26" t="n">
-        <v>392.68</v>
+        <v>269</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>411.12</v>
+        <v>280.51</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>430.26</v>
+        <v>292.44</v>
       </c>
       <c r="G6" s="26" t="n">
-        <v>450.13</v>
+        <v>304.77</v>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="C7" s="26" t="n">
-        <v>250.5</v>
+        <v>205.59</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>262.11</v>
+        <v>214.31</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>274.17</v>
+        <v>223.33</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>286.68</v>
+        <v>232.67</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>299.66</v>
+        <v>242.33</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>8%</t>
         </is>
       </c>
       <c r="C8" s="26" t="n">
-        <v>188.29</v>
+        <v>170.78</v>
       </c>
       <c r="D8" s="26" t="n">
-        <v>196.84</v>
+        <v>177.89</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>205.71</v>
+        <v>185.26</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>214.92</v>
+        <v>192.88</v>
       </c>
       <c r="G8" s="26" t="n">
-        <v>224.46</v>
+        <v>200.76</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>9%</t>
         </is>
       </c>
       <c r="C9" s="26" t="n">
-        <v>150.98</v>
+        <v>145.93</v>
       </c>
       <c r="D9" s="26" t="n">
-        <v>157.69</v>
+        <v>151.91</v>
       </c>
       <c r="E9" s="26" t="n">
-        <v>164.65</v>
+        <v>158.1</v>
       </c>
       <c r="F9" s="26" t="n">
-        <v>171.88</v>
+        <v>164.5</v>
       </c>
       <c r="G9" s="26" t="n">
-        <v>179.36</v>
+        <v>171.11</v>
       </c>
     </row>
   </sheetData>
@@ -1403,16 +1413,16 @@
         <v>-0.01087259597443213</v>
       </c>
       <c r="E5" s="29" t="n">
-        <v>0.3371702737566076</v>
+        <v>0.3371704858923146</v>
       </c>
       <c r="F5" s="28" t="n">
         <v>266.3036468505859</v>
       </c>
       <c r="G5" s="28" t="n">
-        <v>263.8920782470703</v>
+        <v>263.8920809936524</v>
       </c>
       <c r="H5" s="28" t="n">
-        <v>243.5495394897461</v>
+        <v>243.5495402526855</v>
       </c>
       <c r="I5" s="30" t="inlineStr">
         <is>
@@ -1433,16 +1443,16 @@
         <v>0.009399570490431275</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>0.3497391000024921</v>
+        <v>0.3497393141321836</v>
       </c>
       <c r="F6" s="32" t="n">
         <v>265.4054748535156</v>
       </c>
       <c r="G6" s="32" t="n">
-        <v>263.6477954101563</v>
+        <v>263.6477981567383</v>
       </c>
       <c r="H6" s="32" t="n">
-        <v>243.8175304412842</v>
+        <v>243.8175312805176</v>
       </c>
       <c r="I6" s="34" t="inlineStr">
         <is>
@@ -1463,16 +1473,16 @@
         <v>0.003655539804198638</v>
       </c>
       <c r="E7" s="29" t="n">
-        <v>0.3546731250078345</v>
+        <v>0.3546733399202855</v>
       </c>
       <c r="F7" s="28" t="n">
         <v>264.7166091918945</v>
       </c>
       <c r="G7" s="28" t="n">
-        <v>263.3935491943359</v>
+        <v>263.393551940918</v>
       </c>
       <c r="H7" s="28" t="n">
-        <v>244.1140228271484</v>
+        <v>244.1140236663818</v>
       </c>
       <c r="I7" s="30" t="inlineStr">
         <is>
@@ -1493,16 +1503,16 @@
         <v>-7.670678451010549e-05</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>0.354569212388353</v>
+        <v>0.3545694272843187</v>
       </c>
       <c r="F8" s="32" t="n">
         <v>264.0737014770508</v>
       </c>
       <c r="G8" s="32" t="n">
-        <v>263.1470880126953</v>
+        <v>263.1470901489258</v>
       </c>
       <c r="H8" s="32" t="n">
-        <v>244.4140509033203</v>
+        <v>244.4140516662598</v>
       </c>
       <c r="I8" s="34" t="inlineStr">
         <is>
@@ -1523,16 +1533,16 @@
         <v>-0.01936274610273292</v>
       </c>
       <c r="E9" s="29" t="n">
-        <v>0.3283410326502985</v>
+        <v>0.3283412433852881</v>
       </c>
       <c r="F9" s="28" t="n">
         <v>263.0876098632813</v>
       </c>
       <c r="G9" s="28" t="n">
-        <v>262.7925323486328</v>
+        <v>262.7925344848633</v>
       </c>
       <c r="H9" s="28" t="n">
-        <v>244.7191817474365</v>
+        <v>244.7191825866699</v>
       </c>
       <c r="I9" s="30" t="inlineStr">
         <is>
@@ -1553,16 +1563,16 @@
         <v>-0.02205187632814842</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>0.2990486204766891</v>
+        <v>0.2990488265645768</v>
       </c>
       <c r="F10" s="32" t="n">
         <v>262.5076431274414</v>
       </c>
       <c r="G10" s="32" t="n">
-        <v>262.3388562011719</v>
+        <v>262.3388589477539</v>
       </c>
       <c r="H10" s="32" t="n">
-        <v>244.9715362548828</v>
+        <v>244.9715371704102</v>
       </c>
       <c r="I10" s="34" t="inlineStr">
         <is>
@@ -1583,16 +1593,16 @@
         <v>0.01079485974528804</v>
       </c>
       <c r="E11" s="29" t="n">
-        <v>0.3130716681370449</v>
+        <v>0.3130718764496223</v>
       </c>
       <c r="F11" s="28" t="n">
         <v>262.3597801208496</v>
       </c>
       <c r="G11" s="28" t="n">
-        <v>261.9634854125977</v>
+        <v>261.9634881591797</v>
       </c>
       <c r="H11" s="28" t="n">
-        <v>245.2363325500488</v>
+        <v>245.2363334655762</v>
       </c>
       <c r="I11" s="30" t="inlineStr">
         <is>
@@ -1613,16 +1623,16 @@
         <v>0.005577047742174601</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>0.320394731519142</v>
+        <v>0.3203949409934888</v>
       </c>
       <c r="F12" s="32" t="n">
         <v>261.8777236938477</v>
       </c>
       <c r="G12" s="32" t="n">
-        <v>261.6332568359375</v>
+        <v>261.633258972168</v>
       </c>
       <c r="H12" s="32" t="n">
-        <v>245.5105130004883</v>
+        <v>245.5105139923096</v>
       </c>
       <c r="I12" s="34" t="inlineStr">
         <is>
@@ -1643,16 +1653,16 @@
         <v>-0.01687444479508171</v>
       </c>
       <c r="E13" s="29" t="n">
-        <v>0.2981138035144055</v>
+        <v>0.2981140094539889</v>
       </c>
       <c r="F13" s="28" t="n">
         <v>261.157886505127</v>
       </c>
       <c r="G13" s="28" t="n">
-        <v>261.2921682739258</v>
+        <v>261.2921697998047</v>
       </c>
       <c r="H13" s="28" t="n">
-        <v>245.7587809753418</v>
+        <v>245.758782043457</v>
       </c>
       <c r="I13" s="30" t="inlineStr">
         <is>
@@ -1673,16 +1683,16 @@
         <v>-0.003920930967820313</v>
       </c>
       <c r="E14" s="33" t="n">
-        <v>0.2930239889024508</v>
+        <v>0.2930241940345595</v>
       </c>
       <c r="F14" s="32" t="n">
         <v>260.5774230957031</v>
       </c>
       <c r="G14" s="32" t="n">
-        <v>261.02931640625</v>
+        <v>261.0293173217773</v>
       </c>
       <c r="H14" s="32" t="n">
-        <v>245.9979203033447</v>
+        <v>245.99792137146</v>
       </c>
       <c r="I14" s="34" t="inlineStr">
         <is>
@@ -1703,16 +1713,16 @@
         <v>-0.003896244515231628</v>
       </c>
       <c r="E15" s="29" t="n">
-        <v>0.2879860512776267</v>
+        <v>0.2879862556104906</v>
       </c>
       <c r="F15" s="28" t="n">
         <v>259.7486869812012</v>
       </c>
       <c r="G15" s="28" t="n">
-        <v>260.7876071166992</v>
+        <v>260.787607421875</v>
       </c>
       <c r="H15" s="28" t="n">
-        <v>246.2243951416016</v>
+        <v>246.2243962097168</v>
       </c>
       <c r="I15" s="30" t="inlineStr">
         <is>
@@ -1733,16 +1743,16 @@
         <v>0.01411348047549499</v>
       </c>
       <c r="E16" s="33" t="n">
-        <v>0.3061640172650433</v>
+        <v>0.3061642244817553</v>
       </c>
       <c r="F16" s="32" t="n">
         <v>259.0148643493652</v>
       </c>
       <c r="G16" s="32" t="n">
-        <v>260.641584777832</v>
+        <v>260.6415850830078</v>
       </c>
       <c r="H16" s="32" t="n">
-        <v>246.4705949401855</v>
+        <v>246.4705959320068</v>
       </c>
       <c r="I16" s="34" t="inlineStr">
         <is>
@@ -1763,16 +1773,16 @@
         <v>0.0005964238375686381</v>
       </c>
       <c r="E17" s="29" t="n">
-        <v>0.3069430446207146</v>
+        <v>0.3069432519610156</v>
       </c>
       <c r="F17" s="28" t="n">
         <v>257.9908065795898</v>
       </c>
       <c r="G17" s="28" t="n">
-        <v>260.4919720458984</v>
+        <v>260.4919723510742</v>
       </c>
       <c r="H17" s="28" t="n">
-        <v>246.7284506988525</v>
+        <v>246.7284517669678</v>
       </c>
       <c r="I17" s="30" t="inlineStr">
         <is>
@@ -1793,16 +1803,16 @@
         <v>0.003894442556547473</v>
       </c>
       <c r="E18" s="33" t="n">
-        <v>0.3120328592326693</v>
+        <v>0.312033067380445</v>
       </c>
       <c r="F18" s="32" t="n">
         <v>256.9112998962402</v>
       </c>
       <c r="G18" s="32" t="n">
-        <v>260.3443734741211</v>
+        <v>260.3443743896485</v>
       </c>
       <c r="H18" s="32" t="n">
-        <v>246.9748170471191</v>
+        <v>246.9748181152344</v>
       </c>
       <c r="I18" s="34" t="inlineStr">
         <is>
@@ -1823,16 +1833,16 @@
         <v>0.001068833312727335</v>
       </c>
       <c r="E19" s="29" t="n">
-        <v>0.3134352036600101</v>
+        <v>0.3134354120302612</v>
       </c>
       <c r="F19" s="28" t="n">
         <v>255.9092231750488</v>
       </c>
       <c r="G19" s="28" t="n">
-        <v>260.1862002563477</v>
+        <v>260.186201171875</v>
       </c>
       <c r="H19" s="28" t="n">
-        <v>247.2348332977295</v>
+        <v>247.2348345184326</v>
       </c>
       <c r="I19" s="30" t="inlineStr">
         <is>
@@ -1853,16 +1863,16 @@
         <v>-0.01617306867243096</v>
       </c>
       <c r="E20" s="33" t="n">
-        <v>0.2921929259144285</v>
+        <v>0.292193130914693</v>
       </c>
       <c r="F20" s="32" t="n">
         <v>255.1409309387207</v>
       </c>
       <c r="G20" s="32" t="n">
-        <v>259.9680618286133</v>
+        <v>259.9680627441406</v>
       </c>
       <c r="H20" s="32" t="n">
-        <v>247.468342590332</v>
+        <v>247.4683437347412</v>
       </c>
       <c r="I20" s="34" t="inlineStr">
         <is>
@@ -1883,16 +1893,16 @@
         <v>-0.008721851736991693</v>
       </c>
       <c r="E21" s="29" t="n">
-        <v>0.2809226107990133</v>
+        <v>0.280922814011296</v>
       </c>
       <c r="F21" s="28" t="n">
         <v>254.237264251709</v>
       </c>
       <c r="G21" s="28" t="n">
-        <v>259.7414987182617</v>
+        <v>259.7414990234375</v>
       </c>
       <c r="H21" s="28" t="n">
-        <v>247.710384979248</v>
+        <v>247.7103861236572</v>
       </c>
       <c r="I21" s="30" t="inlineStr">
         <is>
@@ -1913,16 +1923,16 @@
         <v>0.02903129041842645</v>
       </c>
       <c r="E22" s="33" t="n">
-        <v>0.3181094471166483</v>
+        <v>0.318109656228446</v>
       </c>
       <c r="F22" s="32" t="n">
         <v>253.7397216796875</v>
       </c>
       <c r="G22" s="32" t="n">
-        <v>259.7115036010742</v>
+        <v>259.7115042114258</v>
       </c>
       <c r="H22" s="32" t="n">
-        <v>247.9861026000977</v>
+        <v>247.9861038208008</v>
       </c>
       <c r="I22" s="34" t="inlineStr">
         <is>
@@ -1943,16 +1953,16 @@
         <v>0.007250134515282447</v>
       </c>
       <c r="E23" s="29" t="n">
-        <v>0.3276659179141086</v>
+        <v>0.3276661285419948</v>
       </c>
       <c r="F23" s="28" t="n">
         <v>253.3955390930176</v>
       </c>
       <c r="G23" s="28" t="n">
-        <v>259.8945474243164</v>
+        <v>259.894548034668</v>
       </c>
       <c r="H23" s="28" t="n">
-        <v>248.2847074890137</v>
+        <v>248.2847087860108</v>
       </c>
       <c r="I23" s="30" t="inlineStr">
         <is>
@@ -1973,16 +1983,16 @@
         <v>0.001134455365532361</v>
       </c>
       <c r="E24" s="33" t="n">
-        <v>0.3291720956383206</v>
+        <v>0.3291723065051548</v>
       </c>
       <c r="F24" s="32" t="n">
         <v>253.1772399902344</v>
       </c>
       <c r="G24" s="32" t="n">
-        <v>260.0644210815429</v>
+        <v>260.0644216918946</v>
       </c>
       <c r="H24" s="32" t="n">
-        <v>248.5749499511719</v>
+        <v>248.5749513244629</v>
       </c>
       <c r="I24" s="34" t="inlineStr">
         <is>
@@ -2003,16 +2013,16 @@
         <v>0.01148787622262004</v>
       </c>
       <c r="E25" s="29" t="n">
-        <v>0.3444414601515742</v>
+        <v>0.3444416734408204</v>
       </c>
       <c r="F25" s="28" t="n">
         <v>253.2471755981445</v>
       </c>
       <c r="G25" s="28" t="n">
-        <v>260.2790661621094</v>
+        <v>260.279066772461</v>
       </c>
       <c r="H25" s="28" t="n">
-        <v>248.8937239074707</v>
+        <v>248.8937252807617</v>
       </c>
       <c r="I25" s="30" t="inlineStr">
         <is>
@@ -2033,16 +2043,16 @@
         <v>-0.0207060792616357</v>
       </c>
       <c r="E26" s="33" t="n">
-        <v>0.3166033487150464</v>
+        <v>0.3166035575879087</v>
       </c>
       <c r="F26" s="32" t="n">
         <v>252.9284698486328</v>
       </c>
       <c r="G26" s="32" t="n">
-        <v>260.3927990722656</v>
+        <v>260.3927996826172</v>
       </c>
       <c r="H26" s="32" t="n">
-        <v>249.1810412597656</v>
+        <v>249.1810425567627</v>
       </c>
       <c r="I26" s="34" t="inlineStr">
         <is>
@@ -2063,16 +2073,16 @@
         <v>0.02130173579070926</v>
       </c>
       <c r="E27" s="29" t="n">
-        <v>0.3446492853905374</v>
+        <v>0.3446494987127542</v>
       </c>
       <c r="F27" s="28" t="n">
         <v>252.8320587158203</v>
       </c>
       <c r="G27" s="28" t="n">
-        <v>260.4673056030273</v>
+        <v>260.4673059082031</v>
       </c>
       <c r="H27" s="28" t="n">
-        <v>249.4733209991455</v>
+        <v>249.4733222198486</v>
       </c>
       <c r="I27" s="30" t="inlineStr">
         <is>
@@ -2093,16 +2103,16 @@
         <v>0.006141348347641795</v>
       </c>
       <c r="E28" s="33" t="n">
-        <v>0.3529072450575284</v>
+        <v>0.3529074596898312</v>
       </c>
       <c r="F28" s="32" t="n">
         <v>252.8160736083984</v>
       </c>
       <c r="G28" s="32" t="n">
-        <v>260.5164895629883</v>
+        <v>260.5164892578125</v>
       </c>
       <c r="H28" s="32" t="n">
-        <v>249.7710531616211</v>
+        <v>249.7710544586182</v>
       </c>
       <c r="I28" s="34" t="inlineStr">
         <is>
@@ -2123,7 +2133,7 @@
         <v>-3.834482173115106e-05</v>
       </c>
       <c r="E29" s="29" t="n">
-        <v>0.3528553680703979</v>
+        <v>0.3528555826944706</v>
       </c>
       <c r="F29" s="28" t="n">
         <v>253.0518569946289</v>
@@ -2132,7 +2142,7 @@
         <v>260.6020050048828</v>
       </c>
       <c r="H29" s="28" t="n">
-        <v>250.0747117614746</v>
+        <v>250.0747130584717</v>
       </c>
       <c r="I29" s="30" t="inlineStr">
         <is>
@@ -2153,7 +2163,7 @@
         <v>-0.004913954203973225</v>
       </c>
       <c r="E30" s="33" t="n">
-        <v>0.3462074987471007</v>
+        <v>0.3462077123165204</v>
       </c>
       <c r="F30" s="32" t="n">
         <v>253.5054397583008</v>
@@ -2162,7 +2172,7 @@
         <v>260.6252130126953</v>
       </c>
       <c r="H30" s="32" t="n">
-        <v>250.3657012176514</v>
+        <v>250.3657025909424</v>
       </c>
       <c r="I30" s="34" t="inlineStr">
         <is>
@@ -2183,16 +2193,16 @@
         <v>-0.00142758690909639</v>
       </c>
       <c r="E31" s="29" t="n">
-        <v>0.344285670544962</v>
+        <v>0.3442858838094927</v>
       </c>
       <c r="F31" s="28" t="n">
         <v>253.8056617736816</v>
       </c>
       <c r="G31" s="28" t="n">
-        <v>260.6170715332031</v>
+        <v>260.6170709228516</v>
       </c>
       <c r="H31" s="28" t="n">
-        <v>250.6576312255859</v>
+        <v>250.657632522583</v>
       </c>
       <c r="I31" s="30" t="inlineStr">
         <is>
@@ -2213,7 +2223,7 @@
         <v>0.02936295529114541</v>
       </c>
       <c r="E32" s="33" t="n">
-        <v>0.3837578705877012</v>
+        <v>0.3837580901143087</v>
       </c>
       <c r="F32" s="32" t="n">
         <v>254.4151000976562</v>
@@ -2222,7 +2232,7 @@
         <v>260.5505804443359</v>
       </c>
       <c r="H32" s="32" t="n">
-        <v>250.9871278381348</v>
+        <v>250.9871291351318</v>
       </c>
       <c r="I32" s="34" t="inlineStr">
         <is>
@@ -2243,7 +2253,7 @@
         <v>-0.01137263363440688</v>
       </c>
       <c r="E33" s="29" t="n">
-        <v>0.3680208992867802</v>
+        <v>0.3680211163167921</v>
       </c>
       <c r="F33" s="28" t="n">
         <v>255.0874794006348</v>
@@ -2252,7 +2262,7 @@
         <v>260.4341253662109</v>
       </c>
       <c r="H33" s="28" t="n">
-        <v>251.2811191558838</v>
+        <v>251.2811204528809</v>
       </c>
       <c r="I33" s="30" t="inlineStr">
         <is>
@@ -2273,7 +2283,7 @@
         <v>0.02593021154924191</v>
       </c>
       <c r="E34" s="33" t="n">
-        <v>0.4034939706090706</v>
+        <v>0.4034941932667166</v>
       </c>
       <c r="F34" s="32" t="n">
         <v>256.15</v>
@@ -2282,7 +2292,7 @@
         <v>260.3142059326172</v>
       </c>
       <c r="H34" s="32" t="n">
-        <v>251.5960314941406</v>
+        <v>251.5960328674316</v>
       </c>
       <c r="I34" s="34" t="inlineStr">
         <is>
@@ -2303,7 +2313,7 @@
         <v>0.01043547537139644</v>
       </c>
       <c r="E35" s="29" t="n">
-        <v>0.418140097373265</v>
+        <v>0.4181403223544493</v>
       </c>
       <c r="F35" s="28" t="n">
         <v>257.4018455505371</v>
@@ -2312,7 +2322,7 @@
         <v>260.2622119140625</v>
       </c>
       <c r="H35" s="28" t="n">
-        <v>251.9020220184326</v>
+        <v>251.9020233917236</v>
       </c>
       <c r="I35" s="30" t="inlineStr">
         <is>
@@ -2333,7 +2343,7 @@
         <v>-0.02519670399569707</v>
       </c>
       <c r="E36" s="33" t="n">
-        <v>0.3824076411153219</v>
+        <v>0.3824078604277219</v>
       </c>
       <c r="F36" s="32" t="n">
         <v>258.1351707458496</v>
@@ -2342,7 +2352,7 @@
         <v>260.0286279296875</v>
       </c>
       <c r="H36" s="32" t="n">
-        <v>252.1681163024902</v>
+        <v>252.1681176757812</v>
       </c>
       <c r="I36" s="34" t="inlineStr">
         <is>
@@ -2363,7 +2373,7 @@
         <v>0.02629899524101398</v>
       </c>
       <c r="E37" s="29" t="n">
-        <v>0.4187635730901551</v>
+        <v>0.4187637981702508</v>
       </c>
       <c r="F37" s="28" t="n">
         <v>259.2106811523437</v>
@@ -2372,7 +2382,7 @@
         <v>259.9996551513672</v>
       </c>
       <c r="H37" s="28" t="n">
-        <v>252.4871073913574</v>
+        <v>252.4871086883545</v>
       </c>
       <c r="I37" s="30" t="inlineStr">
         <is>
@@ -2393,7 +2403,7 @@
         <v>0.0009516944880663125</v>
       </c>
       <c r="E38" s="33" t="n">
-        <v>0.4201138025625342</v>
+        <v>0.4201140278568374</v>
       </c>
       <c r="F38" s="32" t="n">
         <v>260.2502235412597</v>
@@ -2402,7 +2412,7 @@
         <v>259.9946600341797</v>
       </c>
       <c r="H38" s="32" t="n">
-        <v>252.807098236084</v>
+        <v>252.807099609375</v>
       </c>
       <c r="I38" s="34" t="inlineStr">
         <is>
@@ -2423,7 +2433,7 @@
         <v>-0.008667702544387201</v>
       </c>
       <c r="E39" s="29" t="n">
-        <v>0.4078046785427436</v>
+        <v>0.4078049018842627</v>
       </c>
       <c r="F39" s="28" t="n">
         <v>261.157886505127</v>
@@ -2432,7 +2442,7 @@
         <v>259.9059417724609</v>
       </c>
       <c r="H39" s="28" t="n">
-        <v>253.1096222686768</v>
+        <v>253.1096237182617</v>
       </c>
       <c r="I39" s="30" t="inlineStr">
         <is>
@@ -2453,7 +2463,7 @@
         <v>-0.01272786158267403</v>
       </c>
       <c r="E40" s="33" t="n">
-        <v>0.3898863354588107</v>
+        <v>0.3898865559576699</v>
       </c>
       <c r="F40" s="32" t="n">
         <v>262.0975196838379</v>
@@ -2462,7 +2472,7 @@
         <v>260.0234326171875</v>
       </c>
       <c r="H40" s="32" t="n">
-        <v>253.3885872650146</v>
+        <v>253.3885885620117</v>
       </c>
       <c r="I40" s="34" t="inlineStr">
         <is>
@@ -2483,7 +2493,7 @@
         <v>0.01158410276850552</v>
       </c>
       <c r="E41" s="29" t="n">
-        <v>0.4059869216053071</v>
+        <v>0.4059871446584478</v>
       </c>
       <c r="F41" s="28" t="n">
         <v>263.3004112243652</v>
@@ -2492,7 +2502,7 @@
         <v>260.3217578125</v>
       </c>
       <c r="H41" s="28" t="n">
-        <v>253.689263381958</v>
+        <v>253.6892646789551</v>
       </c>
       <c r="I41" s="30" t="inlineStr">
         <is>
@@ -2513,7 +2523,7 @@
         <v>-0.001994705758897597</v>
       </c>
       <c r="E42" s="33" t="n">
-        <v>0.4031823913958463</v>
+        <v>0.4031826140040615</v>
       </c>
       <c r="F42" s="32" t="n">
         <v>264.1186584472656</v>
@@ -2522,7 +2532,7 @@
         <v>260.4474420166015</v>
       </c>
       <c r="H42" s="32" t="n">
-        <v>253.9998918914795</v>
+        <v>253.9998931121826</v>
       </c>
       <c r="I42" s="34" t="inlineStr">
         <is>
@@ -2543,7 +2553,7 @@
         <v>0.004367659937802859</v>
       </c>
       <c r="E43" s="29" t="n">
-        <v>0.4093110149121764</v>
+        <v>0.4093112384926685</v>
       </c>
       <c r="F43" s="28" t="n">
         <v>264.9039360046387</v>
@@ -2552,7 +2562,7 @@
         <v>260.5873132324219</v>
       </c>
       <c r="H43" s="28" t="n">
-        <v>254.313974609375</v>
+        <v>254.3139758300781</v>
       </c>
       <c r="I43" s="30" t="inlineStr">
         <is>
@@ -2573,7 +2583,7 @@
         <v>0.03239351812191993</v>
       </c>
       <c r="E44" s="33" t="n">
-        <v>0.4549635568131554</v>
+        <v>0.4549637876362063</v>
       </c>
       <c r="F44" s="32" t="n">
         <v>266.1138214111328</v>
@@ -2582,7 +2592,7 @@
         <v>260.9781536865235</v>
       </c>
       <c r="H44" s="32" t="n">
-        <v>254.6667375183106</v>
+        <v>254.6667388153076</v>
       </c>
       <c r="I44" s="34" t="inlineStr">
         <is>
@@ -2603,7 +2613,7 @@
         <v>-0.01181560318641728</v>
       </c>
       <c r="E45" s="29" t="n">
-        <v>0.4377722847751528</v>
+        <v>0.4377725128708903</v>
       </c>
       <c r="F45" s="28" t="n">
         <v>267.0114944458008</v>
@@ -2612,7 +2622,7 @@
         <v>261.2229278564453</v>
       </c>
       <c r="H45" s="28" t="n">
-        <v>255.0036628723145</v>
+        <v>255.0036640930176</v>
       </c>
       <c r="I45" s="30" t="inlineStr">
         <is>
@@ -2633,7 +2643,7 @@
         <v>0.02655069092770845</v>
       </c>
       <c r="E46" s="33" t="n">
-        <v>0.475946132332643</v>
+        <v>0.4759463664844801</v>
       </c>
       <c r="F46" s="32" t="n">
         <v>268.5440826416016</v>
@@ -2642,7 +2652,7 @@
         <v>261.5825970458984</v>
       </c>
       <c r="H46" s="32" t="n">
-        <v>255.3715274810791</v>
+        <v>255.3715286254883</v>
       </c>
       <c r="I46" s="34" t="inlineStr">
         <is>
@@ -2663,7 +2673,7 @@
         <v>0.01171792495226764</v>
       </c>
       <c r="E47" s="29" t="n">
-        <v>0.4932411583449066</v>
+        <v>0.4932413952405172</v>
       </c>
       <c r="F47" s="28" t="n">
         <v>269.9732666015625</v>
@@ -2672,7 +2682,7 @@
         <v>261.8897137451172</v>
       </c>
       <c r="H47" s="28" t="n">
-        <v>255.7495524597168</v>
+        <v>255.749553604126</v>
       </c>
       <c r="I47" s="30" t="inlineStr">
         <is>
@@ -2693,7 +2703,7 @@
         <v>-0.0002435071144024636</v>
       </c>
       <c r="E48" s="33" t="n">
-        <v>0.4928775434993311</v>
+        <v>0.4928777803372559</v>
       </c>
       <c r="F48" s="32" t="n">
         <v>271.3195266723633</v>
@@ -2702,7 +2712,7 @@
         <v>262.1536700439453</v>
       </c>
       <c r="H48" s="32" t="n">
-        <v>256.1176655578613</v>
+        <v>256.1176667785645</v>
       </c>
       <c r="I48" s="34" t="inlineStr">
         <is>
@@ -2723,7 +2733,7 @@
         <v>0.02045649788887838</v>
       </c>
       <c r="E49" s="29" t="n">
-        <v>0.523416589816279</v>
+        <v>0.5234168314990784</v>
       </c>
       <c r="F49" s="28" t="n">
         <v>272.9600158691406</v>
@@ -2732,7 +2742,7 @@
         <v>262.5606951904297</v>
       </c>
       <c r="H49" s="28" t="n">
-        <v>256.5163967132568</v>
+        <v>256.51639793396</v>
       </c>
       <c r="I49" s="30" t="inlineStr">
         <is>
@@ -2753,7 +2763,7 @@
         <v>-0.001262670573777269</v>
       </c>
       <c r="E50" s="33" t="n">
-        <v>0.521493016516714</v>
+        <v>0.5214932578943474</v>
       </c>
       <c r="F50" s="32" t="n">
         <v>274.6459442138672</v>
@@ -2762,7 +2772,7 @@
         <v>263.1355584716797</v>
       </c>
       <c r="H50" s="32" t="n">
-        <v>256.9152201843262</v>
+        <v>256.9152213287354</v>
       </c>
       <c r="I50" s="34" t="inlineStr">
         <is>
@@ -2783,7 +2793,7 @@
         <v>0.007243389265544797</v>
       </c>
       <c r="E51" s="29" t="n">
-        <v>0.5325137827001525</v>
+        <v>0.532514025826178</v>
       </c>
       <c r="F51" s="28" t="n">
         <v>276.4563568115234</v>
@@ -2792,7 +2802,7 @@
         <v>263.7420318603516</v>
       </c>
       <c r="H51" s="28" t="n">
-        <v>257.3240458679199</v>
+        <v>257.3240469360351</v>
       </c>
       <c r="I51" s="30" t="inlineStr">
         <is>
@@ -2813,7 +2823,7 @@
         <v>0.01380599556563422</v>
       </c>
       <c r="E52" s="33" t="n">
-        <v>0.5536716611883841</v>
+        <v>0.5536719076710064</v>
       </c>
       <c r="F52" s="32" t="n">
         <v>278.0906188964844</v>
@@ -2822,7 +2832,7 @@
         <v>264.449287109375</v>
       </c>
       <c r="H52" s="32" t="n">
-        <v>257.7523748779297</v>
+        <v>257.7523760223389</v>
       </c>
       <c r="I52" s="34" t="inlineStr">
         <is>
@@ -2843,7 +2853,7 @@
         <v>-0.00220833028705536</v>
       </c>
       <c r="E53" s="29" t="n">
-        <v>0.5502406410028422</v>
+        <v>0.5502408869411495</v>
       </c>
       <c r="F53" s="28" t="n">
         <v>279.8432418823242</v>
@@ -2852,7 +2862,7 @@
         <v>265.167919921875</v>
       </c>
       <c r="H53" s="28" t="n">
-        <v>258.1912490081787</v>
+        <v>258.1912502288818</v>
       </c>
       <c r="I53" s="30" t="inlineStr">
         <is>
@@ -2873,7 +2883,7 @@
         <v>0.006773815730967137</v>
       </c>
       <c r="E54" s="33" t="n">
-        <v>0.5607416854436518</v>
+        <v>0.5607419330479</v>
       </c>
       <c r="F54" s="32" t="n">
         <v>281.3556793212891</v>
@@ -2882,7 +2892,7 @@
         <v>265.9715118408203</v>
       </c>
       <c r="H54" s="32" t="n">
-        <v>258.6512794494629</v>
+        <v>258.651280670166</v>
       </c>
       <c r="I54" s="34" t="inlineStr">
         <is>
@@ -2903,7 +2913,7 @@
         <v>-0.007960612067346995</v>
       </c>
       <c r="E55" s="29" t="n">
-        <v>0.5483172263484974</v>
+        <v>0.5483174719816644</v>
       </c>
       <c r="F55" s="28" t="n">
         <v>282.607746887207</v>
@@ -2912,7 +2922,7 @@
         <v>266.7838519287109</v>
       </c>
       <c r="H55" s="28" t="n">
-        <v>259.1067304992676</v>
+        <v>259.1067316436768</v>
       </c>
       <c r="I55" s="30" t="inlineStr">
         <is>
@@ -2933,7 +2943,7 @@
         <v>0.003793999787491842</v>
       </c>
       <c r="E56" s="33" t="n">
-        <v>0.5541915415762335</v>
+        <v>0.5541917881413327</v>
       </c>
       <c r="F56" s="32" t="n">
         <v>284.2599960327149</v>
@@ -2942,7 +2952,7 @@
         <v>267.5704364013672</v>
       </c>
       <c r="H56" s="32" t="n">
-        <v>259.5936789703369</v>
+        <v>259.5936801910401</v>
       </c>
       <c r="I56" s="34" t="inlineStr">
         <is>
@@ -2963,7 +2973,7 @@
         <v>0.0109709963070026</v>
       </c>
       <c r="E57" s="29" t="n">
-        <v>0.571242571239241</v>
+        <v>0.5712428205094051</v>
       </c>
       <c r="F57" s="28" t="n">
         <v>285.7265670776367</v>
@@ -2972,7 +2982,7 @@
         <v>268.4036383056641</v>
       </c>
       <c r="H57" s="28" t="n">
-        <v>260.0921966552734</v>
+        <v>260.0921978759766</v>
       </c>
       <c r="I57" s="30" t="inlineStr">
         <is>
@@ -2993,7 +3003,7 @@
         <v>0.009065310949131433</v>
       </c>
       <c r="E58" s="33" t="n">
-        <v>0.5854863737240377</v>
+        <v>0.5854866252539133</v>
       </c>
       <c r="F58" s="32" t="n">
         <v>287.3171508789063</v>
@@ -3002,7 +3012,7 @@
         <v>269.2920397949219</v>
       </c>
       <c r="H58" s="32" t="n">
-        <v>260.6065558624268</v>
+        <v>260.6065571594238</v>
       </c>
       <c r="I58" s="34" t="inlineStr">
         <is>
@@ -3023,7 +3033,7 @@
         <v>0.01255784521616765</v>
       </c>
       <c r="E59" s="29" t="n">
-        <v>0.6053966661976071</v>
+        <v>0.6053969208861558</v>
       </c>
       <c r="F59" s="28" t="n">
         <v>289.217626953125</v>
@@ -3032,7 +3042,7 @@
         <v>270.3579486083984</v>
       </c>
       <c r="H59" s="28" t="n">
-        <v>261.0886191558838</v>
+        <v>261.0886205291748</v>
       </c>
       <c r="I59" s="30" t="inlineStr">
         <is>
@@ -3053,7 +3063,7 @@
         <v>-0.001586751960143129</v>
       </c>
       <c r="E60" s="33" t="n">
-        <v>0.6028492998907109</v>
+        <v>0.602849554175132</v>
       </c>
       <c r="F60" s="32" t="n">
         <v>291.2659439086914</v>
@@ -3062,7 +3072,7 @@
         <v>271.5267529296875</v>
       </c>
       <c r="H60" s="32" t="n">
-        <v>261.5344664001465</v>
+        <v>261.5344676971436</v>
       </c>
       <c r="I60" s="34" t="inlineStr">
         <is>
@@ -3083,7 +3093,7 @@
         <v>0.008173125031610828</v>
       </c>
       <c r="E61" s="29" t="n">
-        <v>0.6159495876255476</v>
+        <v>0.6159498439882669</v>
       </c>
       <c r="F61" s="28" t="n">
         <v>293.2854034423828</v>
@@ -3092,7 +3102,7 @@
         <v>272.6920071411133</v>
       </c>
       <c r="H61" s="28" t="n">
-        <v>261.9464978027344</v>
+        <v>261.9464990234375</v>
       </c>
       <c r="I61" s="30" t="inlineStr">
         <is>
@@ -3113,7 +3123,7 @@
         <v>0.005340207912225559</v>
       </c>
       <c r="E62" s="33" t="n">
-        <v>0.6245790943991432</v>
+        <v>0.6245793521308927</v>
       </c>
       <c r="F62" s="32" t="n">
         <v>295.4148376464844</v>
@@ -3122,7 +3132,7 @@
         <v>273.8622875976562</v>
       </c>
       <c r="H62" s="32" t="n">
-        <v>262.3763523864746</v>
+        <v>262.3763536071777</v>
       </c>
       <c r="I62" s="34" t="inlineStr">
         <is>
@@ -3143,7 +3153,7 @@
         <v>-0.001439992937726231</v>
       </c>
       <c r="E63" s="29" t="n">
-        <v>0.6222397119764307</v>
+        <v>0.6222399693370484</v>
       </c>
       <c r="F63" s="28" t="n">
         <v>297.462825012207</v>
@@ -3152,7 +3162,7 @@
         <v>275.1092886352539</v>
       </c>
       <c r="H63" s="28" t="n">
-        <v>262.7916417694092</v>
+        <v>262.7916429901123</v>
       </c>
       <c r="I63" s="30" t="inlineStr">
         <is>
@@ -3173,7 +3183,7 @@
         <v>-0.01842594387292573</v>
       </c>
       <c r="E64" s="33" t="n">
-        <v>0.5923484140951218</v>
+        <v>0.5923486667136271</v>
       </c>
       <c r="F64" s="32" t="n">
         <v>298.7842178344727</v>
@@ -3182,7 +3192,7 @@
         <v>276.2608715820313</v>
       </c>
       <c r="H64" s="32" t="n">
-        <v>263.1598329925537</v>
+        <v>263.1598342132568</v>
       </c>
       <c r="I64" s="34" t="inlineStr">
         <is>

</xml_diff>